<commit_message>
📊 BIST Screener | 28.05.2026 18:22 | 611 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-28.xlsx
+++ b/data/bist_screener_2026-05-28.xlsx
@@ -13719,42 +13719,44 @@
     <row r="305">
       <c r="A305" s="6" t="inlineStr">
         <is>
-          <t>DAGI</t>
+          <t>TURGG</t>
         </is>
       </c>
       <c r="B305" s="7" t="n">
-        <v>6.78</v>
+        <v>30.42</v>
       </c>
       <c r="C305" s="8" t="n">
-        <v>-0.0231</v>
+        <v>-0.0026</v>
       </c>
       <c r="D305" s="9" t="n">
-        <v>7950000</v>
+        <v>661000</v>
       </c>
       <c r="E305" s="8" t="n">
-        <v>0.4383</v>
+        <v>0.2511</v>
       </c>
       <c r="F305" s="7" t="n">
-        <v>53.46</v>
-      </c>
-      <c r="G305" s="6" t="inlineStr"/>
+        <v>37.19</v>
+      </c>
+      <c r="G305" s="7" t="n">
+        <v>18.23</v>
+      </c>
       <c r="H305" s="7" t="n">
-        <v>1.62</v>
+        <v>1.6</v>
       </c>
       <c r="I305" s="8" t="n">
-        <v>-0.1117</v>
+        <v>0.0842</v>
       </c>
       <c r="J305" s="8" t="n">
-        <v>6.849</v>
+        <v>-1.0919</v>
       </c>
       <c r="K305" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L305" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TEKSTİL DERİ, BIST İSTANBUL, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M305" s="6" t="inlineStr"/>
@@ -13762,42 +13764,42 @@
     <row r="306">
       <c r="A306" s="2" t="inlineStr">
         <is>
-          <t>YAYLA</t>
+          <t>DAGI</t>
         </is>
       </c>
       <c r="B306" s="3" t="n">
-        <v>26.74</v>
+        <v>6.78</v>
       </c>
       <c r="C306" s="4" t="n">
-        <v>-0.0234</v>
+        <v>-0.0231</v>
       </c>
       <c r="D306" s="5" t="n">
-        <v>2340000</v>
+        <v>7950000</v>
       </c>
       <c r="E306" s="4" t="n">
-        <v>0.3133</v>
+        <v>0.4383</v>
       </c>
       <c r="F306" s="3" t="n">
-        <v>49.54</v>
+        <v>53.46</v>
       </c>
       <c r="G306" s="2" t="inlineStr"/>
       <c r="H306" s="3" t="n">
         <v>1.62</v>
       </c>
       <c r="I306" s="4" t="n">
-        <v>-0.01</v>
+        <v>-0.1117</v>
       </c>
       <c r="J306" s="4" t="n">
-        <v>0.0576</v>
+        <v>6.849</v>
       </c>
       <c r="K306" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L306" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HİZMETLER, BIST ANA, BIST ANKARA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TEKSTİL DERİ, BIST İSTANBUL, BIST ANA</t>
         </is>
       </c>
       <c r="M306" s="2" t="inlineStr"/>
@@ -13805,44 +13807,42 @@
     <row r="307">
       <c r="A307" s="6" t="inlineStr">
         <is>
-          <t>TEZOL</t>
+          <t>YAYLA</t>
         </is>
       </c>
       <c r="B307" s="7" t="n">
-        <v>19.65</v>
+        <v>26.74</v>
       </c>
       <c r="C307" s="8" t="n">
-        <v>0.04019999999999999</v>
+        <v>-0.0234</v>
       </c>
       <c r="D307" s="9" t="n">
-        <v>5510000</v>
+        <v>2340000</v>
       </c>
       <c r="E307" s="8" t="n">
-        <v>0.2393</v>
+        <v>0.3133</v>
       </c>
       <c r="F307" s="7" t="n">
-        <v>59.76</v>
-      </c>
-      <c r="G307" s="7" t="n">
-        <v>55.03</v>
-      </c>
+        <v>49.54</v>
+      </c>
+      <c r="G307" s="6" t="inlineStr"/>
       <c r="H307" s="7" t="n">
         <v>1.62</v>
       </c>
       <c r="I307" s="8" t="n">
-        <v>0.0336</v>
+        <v>-0.01</v>
       </c>
       <c r="J307" s="8" t="n">
-        <v>-1.3921</v>
+        <v>0.0576</v>
       </c>
       <c r="K307" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L307" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HİZMETLER, BIST ANA, BIST ANKARA</t>
         </is>
       </c>
       <c r="M307" s="6" t="inlineStr"/>
@@ -13850,128 +13850,128 @@
     <row r="308">
       <c r="A308" s="2" t="inlineStr">
         <is>
-          <t>YONGA</t>
+          <t>TEZOL</t>
         </is>
       </c>
       <c r="B308" s="3" t="n">
-        <v>59</v>
+        <v>19.65</v>
       </c>
       <c r="C308" s="4" t="n">
-        <v>0.0351</v>
+        <v>0.04019999999999999</v>
       </c>
       <c r="D308" s="5" t="n">
-        <v>19650</v>
+        <v>5510000</v>
       </c>
       <c r="E308" s="4" t="n">
-        <v>0.5162</v>
+        <v>0.2393</v>
       </c>
       <c r="F308" s="3" t="n">
-        <v>55.82</v>
+        <v>59.76</v>
       </c>
       <c r="G308" s="3" t="n">
-        <v>207.67</v>
+        <v>55.03</v>
       </c>
       <c r="H308" s="3" t="n">
-        <v>1.64</v>
+        <v>1.62</v>
       </c>
       <c r="I308" s="4" t="n">
-        <v>0.009000000000000001</v>
-      </c>
-      <c r="J308" s="2" t="inlineStr"/>
+        <v>0.0336</v>
+      </c>
+      <c r="J308" s="4" t="n">
+        <v>-1.3921</v>
+      </c>
       <c r="K308" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
-        </is>
-      </c>
-      <c r="L308" s="2" t="inlineStr"/>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
+        </is>
+      </c>
+      <c r="L308" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST İZMİR</t>
+        </is>
+      </c>
       <c r="M308" s="2" t="inlineStr"/>
     </row>
     <row r="309">
       <c r="A309" s="6" t="inlineStr">
         <is>
-          <t>RYSAS</t>
+          <t>YONGA</t>
         </is>
       </c>
       <c r="B309" s="7" t="n">
-        <v>22.2</v>
+        <v>59</v>
       </c>
       <c r="C309" s="8" t="n">
-        <v>0.099</v>
+        <v>0.0351</v>
       </c>
       <c r="D309" s="9" t="n">
-        <v>13230000</v>
+        <v>19650</v>
       </c>
       <c r="E309" s="8" t="n">
-        <v>0.5734</v>
+        <v>0.5162</v>
       </c>
       <c r="F309" s="7" t="n">
-        <v>64.28</v>
+        <v>55.82</v>
       </c>
       <c r="G309" s="7" t="n">
-        <v>13.34</v>
+        <v>207.67</v>
       </c>
       <c r="H309" s="7" t="n">
         <v>1.64</v>
       </c>
       <c r="I309" s="8" t="n">
-        <v>0.1477</v>
-      </c>
-      <c r="J309" s="8" t="n">
-        <v>-0.8042</v>
-      </c>
+        <v>0.009000000000000001</v>
+      </c>
+      <c r="J309" s="6" t="inlineStr"/>
       <c r="K309" s="6" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L309" s="6" t="inlineStr">
-        <is>
-          <t>BIST ULASTIRMA, BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
-        </is>
-      </c>
+          <t>Dayanıklı tüketim malları</t>
+        </is>
+      </c>
+      <c r="L309" s="6" t="inlineStr"/>
       <c r="M309" s="6" t="inlineStr"/>
     </row>
     <row r="310">
       <c r="A310" s="2" t="inlineStr">
         <is>
-          <t>SKBNK</t>
+          <t>RYSAS</t>
         </is>
       </c>
       <c r="B310" s="3" t="n">
-        <v>13.17</v>
+        <v>22.2</v>
       </c>
       <c r="C310" s="4" t="n">
-        <v>-0.0323</v>
+        <v>0.099</v>
       </c>
       <c r="D310" s="5" t="n">
-        <v>28640000</v>
+        <v>13230000</v>
       </c>
       <c r="E310" s="4" t="n">
-        <v>0.5033</v>
+        <v>0.5734</v>
       </c>
       <c r="F310" s="3" t="n">
-        <v>49.82</v>
+        <v>64.28</v>
       </c>
       <c r="G310" s="3" t="n">
-        <v>12.07</v>
+        <v>13.34</v>
       </c>
       <c r="H310" s="3" t="n">
         <v>1.64</v>
       </c>
       <c r="I310" s="4" t="n">
-        <v>0.1501</v>
+        <v>0.1477</v>
       </c>
       <c r="J310" s="4" t="n">
-        <v>-0.1255</v>
+        <v>-0.8042</v>
       </c>
       <c r="K310" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Taşımacılık</t>
         </is>
       </c>
       <c r="L310" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST BANKA, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST MALİ, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST ULASTIRMA, BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M310" s="2" t="inlineStr"/>
@@ -13979,42 +13979,44 @@
     <row r="311">
       <c r="A311" s="6" t="inlineStr">
         <is>
-          <t>OZYSR</t>
+          <t>SKBNK</t>
         </is>
       </c>
       <c r="B311" s="7" t="n">
-        <v>11.79</v>
+        <v>13.17</v>
       </c>
       <c r="C311" s="8" t="n">
-        <v>-0.0008</v>
+        <v>-0.0323</v>
       </c>
       <c r="D311" s="9" t="n">
-        <v>2930000</v>
+        <v>28640000</v>
       </c>
       <c r="E311" s="8" t="n">
-        <v>0.2862</v>
+        <v>0.5033</v>
       </c>
       <c r="F311" s="7" t="n">
-        <v>46.9</v>
-      </c>
-      <c r="G311" s="6" t="inlineStr"/>
+        <v>49.82</v>
+      </c>
+      <c r="G311" s="7" t="n">
+        <v>12.07</v>
+      </c>
       <c r="H311" s="7" t="n">
-        <v>1.66</v>
+        <v>1.64</v>
       </c>
       <c r="I311" s="8" t="n">
-        <v>-0.08710000000000001</v>
+        <v>0.1501</v>
       </c>
       <c r="J311" s="8" t="n">
-        <v>-17.9959</v>
+        <v>-0.1255</v>
       </c>
       <c r="K311" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L311" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST 100, BIST BANKA, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST MALİ, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M311" s="6" t="inlineStr"/>
@@ -14022,40 +14024,42 @@
     <row r="312">
       <c r="A312" s="2" t="inlineStr">
         <is>
-          <t>DNISI</t>
+          <t>OZYSR</t>
         </is>
       </c>
       <c r="B312" s="3" t="n">
-        <v>19.33</v>
+        <v>11.79</v>
       </c>
       <c r="C312" s="4" t="n">
-        <v>-0.0015</v>
+        <v>-0.0008</v>
       </c>
       <c r="D312" s="5" t="n">
-        <v>1180000</v>
-      </c>
-      <c r="E312" s="2" t="inlineStr"/>
+        <v>2930000</v>
+      </c>
+      <c r="E312" s="4" t="n">
+        <v>0.2862</v>
+      </c>
       <c r="F312" s="3" t="n">
-        <v>43.31</v>
-      </c>
-      <c r="G312" s="3" t="n">
-        <v>81.15000000000001</v>
-      </c>
+        <v>46.9</v>
+      </c>
+      <c r="G312" s="2" t="inlineStr"/>
       <c r="H312" s="3" t="n">
-        <v>1.67</v>
+        <v>1.66</v>
       </c>
       <c r="I312" s="4" t="n">
-        <v>0.0235</v>
-      </c>
-      <c r="J312" s="2" t="inlineStr"/>
+        <v>-0.08710000000000001</v>
+      </c>
+      <c r="J312" s="4" t="n">
+        <v>-17.9959</v>
+      </c>
       <c r="K312" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L312" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST KATILIM TÜM, BIST ANA, BIST KOBİ SANAYİ, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M312" s="2" t="inlineStr"/>
@@ -14063,128 +14067,124 @@
     <row r="313">
       <c r="A313" s="6" t="inlineStr">
         <is>
-          <t>AYES</t>
+          <t>DNISI</t>
         </is>
       </c>
       <c r="B313" s="7" t="n">
-        <v>33.98</v>
+        <v>19.33</v>
       </c>
       <c r="C313" s="8" t="n">
-        <v>0.0645</v>
+        <v>-0.0015</v>
       </c>
       <c r="D313" s="9" t="n">
-        <v>202690</v>
-      </c>
-      <c r="E313" s="8" t="n">
-        <v>0.9654</v>
-      </c>
+        <v>1180000</v>
+      </c>
+      <c r="E313" s="6" t="inlineStr"/>
       <c r="F313" s="7" t="n">
-        <v>71.36</v>
+        <v>43.31</v>
       </c>
       <c r="G313" s="7" t="n">
-        <v>4.95</v>
+        <v>81.15000000000001</v>
       </c>
       <c r="H313" s="7" t="n">
-        <v>1.68</v>
+        <v>1.67</v>
       </c>
       <c r="I313" s="8" t="n">
-        <v>0.4496</v>
+        <v>0.0235</v>
       </c>
       <c r="J313" s="6" t="inlineStr"/>
       <c r="K313" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L313" s="6" t="inlineStr"/>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L313" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST KATILIM TÜM, BIST ANA, BIST KOBİ SANAYİ, BIST İZMİR</t>
+        </is>
+      </c>
       <c r="M313" s="6" t="inlineStr"/>
     </row>
     <row r="314">
       <c r="A314" s="2" t="inlineStr">
         <is>
-          <t>MERCN</t>
+          <t>AYES</t>
         </is>
       </c>
       <c r="B314" s="3" t="n">
-        <v>21.5</v>
+        <v>33.98</v>
       </c>
       <c r="C314" s="4" t="n">
-        <v>0.0132</v>
+        <v>0.0645</v>
       </c>
       <c r="D314" s="5" t="n">
-        <v>6170000</v>
+        <v>202690</v>
       </c>
       <c r="E314" s="4" t="n">
-        <v>0.3908</v>
+        <v>0.9654</v>
       </c>
       <c r="F314" s="3" t="n">
-        <v>49.44</v>
+        <v>71.36</v>
       </c>
       <c r="G314" s="3" t="n">
-        <v>30.33</v>
+        <v>4.95</v>
       </c>
       <c r="H314" s="3" t="n">
         <v>1.68</v>
       </c>
       <c r="I314" s="4" t="n">
-        <v>0.0639</v>
-      </c>
-      <c r="J314" s="4" t="n">
-        <v>0.2738</v>
-      </c>
+        <v>0.4496</v>
+      </c>
+      <c r="J314" s="2" t="inlineStr"/>
       <c r="K314" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L314" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST DENİZLİ</t>
-        </is>
-      </c>
+          <t>Üretici imalatı</t>
+        </is>
+      </c>
+      <c r="L314" s="2" t="inlineStr"/>
       <c r="M314" s="2" t="inlineStr"/>
     </row>
     <row r="315">
       <c r="A315" s="6" t="inlineStr">
         <is>
-          <t>DERHL</t>
+          <t>MERCN</t>
         </is>
       </c>
       <c r="B315" s="7" t="n">
-        <v>14.52</v>
+        <v>21.5</v>
       </c>
       <c r="C315" s="8" t="n">
-        <v>0.0083</v>
+        <v>0.0132</v>
       </c>
       <c r="D315" s="9" t="n">
-        <v>4250000</v>
+        <v>6170000</v>
       </c>
       <c r="E315" s="8" t="n">
-        <v>0.2169</v>
+        <v>0.3908</v>
       </c>
       <c r="F315" s="7" t="n">
-        <v>47.53</v>
+        <v>49.44</v>
       </c>
       <c r="G315" s="7" t="n">
-        <v>370.41</v>
+        <v>30.33</v>
       </c>
       <c r="H315" s="7" t="n">
         <v>1.68</v>
       </c>
       <c r="I315" s="8" t="n">
-        <v>0.0051</v>
+        <v>0.0639</v>
       </c>
       <c r="J315" s="8" t="n">
-        <v>-3.014</v>
+        <v>0.2738</v>
       </c>
       <c r="K315" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L315" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST İSTANBUL, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST DENİZLİ</t>
         </is>
       </c>
       <c r="M315" s="6" t="inlineStr"/>
@@ -14192,126 +14192,128 @@
     <row r="316">
       <c r="A316" s="2" t="inlineStr">
         <is>
-          <t>CMENT</t>
+          <t>DERHL</t>
         </is>
       </c>
       <c r="B316" s="3" t="n">
-        <v>309</v>
+        <v>14.52</v>
       </c>
       <c r="C316" s="4" t="n">
-        <v>0.0334</v>
+        <v>0.0083</v>
       </c>
       <c r="D316" s="5" t="n">
-        <v>7950</v>
+        <v>4250000</v>
       </c>
       <c r="E316" s="4" t="n">
-        <v>0.0067</v>
+        <v>0.2169</v>
       </c>
       <c r="F316" s="3" t="n">
-        <v>45.06</v>
+        <v>47.53</v>
       </c>
       <c r="G316" s="3" t="n">
-        <v>22.45</v>
+        <v>370.41</v>
       </c>
       <c r="H316" s="3" t="n">
-        <v>1.69</v>
+        <v>1.68</v>
       </c>
       <c r="I316" s="4" t="n">
-        <v>0.0885</v>
+        <v>0.0051</v>
       </c>
       <c r="J316" s="4" t="n">
-        <v>-0.0863</v>
+        <v>-3.014</v>
       </c>
       <c r="K316" s="2" t="inlineStr">
         <is>
-          <t>Enerji-dışı mineraller</t>
-        </is>
-      </c>
-      <c r="L316" s="2" t="inlineStr"/>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
+        </is>
+      </c>
+      <c r="L316" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST İSTANBUL, BIST ANA</t>
+        </is>
+      </c>
       <c r="M316" s="2" t="inlineStr"/>
     </row>
     <row r="317">
       <c r="A317" s="6" t="inlineStr">
         <is>
-          <t>JANTS</t>
+          <t>CMENT</t>
         </is>
       </c>
       <c r="B317" s="7" t="n">
-        <v>17.35</v>
+        <v>309</v>
       </c>
       <c r="C317" s="8" t="n">
-        <v>-0.0142</v>
+        <v>0.0334</v>
       </c>
       <c r="D317" s="9" t="n">
-        <v>4910000</v>
+        <v>7950</v>
       </c>
       <c r="E317" s="8" t="n">
-        <v>0.2094</v>
+        <v>0.0067</v>
       </c>
       <c r="F317" s="7" t="n">
-        <v>47.26</v>
-      </c>
-      <c r="G317" s="6" t="inlineStr"/>
+        <v>45.06</v>
+      </c>
+      <c r="G317" s="7" t="n">
+        <v>22.45</v>
+      </c>
       <c r="H317" s="7" t="n">
-        <v>1.7</v>
+        <v>1.69</v>
       </c>
       <c r="I317" s="8" t="n">
-        <v>-0.0174</v>
+        <v>0.0885</v>
       </c>
       <c r="J317" s="8" t="n">
-        <v>-1.6348</v>
+        <v>-0.0863</v>
       </c>
       <c r="K317" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L317" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST KATILIM TEMETTU, BIST AYDIN</t>
-        </is>
-      </c>
+          <t>Enerji-dışı mineraller</t>
+        </is>
+      </c>
+      <c r="L317" s="6" t="inlineStr"/>
       <c r="M317" s="6" t="inlineStr"/>
     </row>
     <row r="318">
       <c r="A318" s="2" t="inlineStr">
         <is>
-          <t>KOPOL</t>
+          <t>JANTS</t>
         </is>
       </c>
       <c r="B318" s="3" t="n">
-        <v>6.08</v>
+        <v>17.35</v>
       </c>
       <c r="C318" s="4" t="n">
-        <v>0.0393</v>
+        <v>-0.0142</v>
       </c>
       <c r="D318" s="5" t="n">
-        <v>19190000</v>
+        <v>4910000</v>
       </c>
       <c r="E318" s="4" t="n">
-        <v>0.3854</v>
+        <v>0.2094</v>
       </c>
       <c r="F318" s="3" t="n">
-        <v>51.34</v>
+        <v>47.26</v>
       </c>
       <c r="G318" s="2" t="inlineStr"/>
       <c r="H318" s="3" t="n">
-        <v>1.71</v>
+        <v>1.7</v>
       </c>
       <c r="I318" s="4" t="n">
-        <v>-0.0104</v>
+        <v>-0.0174</v>
       </c>
       <c r="J318" s="4" t="n">
-        <v>-2.9114</v>
+        <v>-1.6348</v>
       </c>
       <c r="K318" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L318" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST KATILIM TEMETTU, BIST AYDIN</t>
         </is>
       </c>
       <c r="M318" s="2" t="inlineStr"/>
@@ -14319,42 +14321,42 @@
     <row r="319">
       <c r="A319" s="6" t="inlineStr">
         <is>
-          <t>HOROZ</t>
+          <t>KOPOL</t>
         </is>
       </c>
       <c r="B319" s="7" t="n">
-        <v>71.75</v>
+        <v>6.08</v>
       </c>
       <c r="C319" s="8" t="n">
-        <v>0.0235</v>
+        <v>0.0393</v>
       </c>
       <c r="D319" s="9" t="n">
-        <v>3740000</v>
+        <v>19190000</v>
       </c>
       <c r="E319" s="8" t="n">
-        <v>0.8178</v>
+        <v>0.3854</v>
       </c>
       <c r="F319" s="7" t="n">
-        <v>47.14</v>
+        <v>51.34</v>
       </c>
       <c r="G319" s="6" t="inlineStr"/>
       <c r="H319" s="7" t="n">
-        <v>1.73</v>
+        <v>1.71</v>
       </c>
       <c r="I319" s="8" t="n">
-        <v>-0.0183</v>
+        <v>-0.0104</v>
       </c>
       <c r="J319" s="8" t="n">
-        <v>-2.2684</v>
+        <v>-2.9114</v>
       </c>
       <c r="K319" s="6" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L319" s="6" t="inlineStr">
         <is>
-          <t>BIST ULASTIRMA, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M319" s="6" t="inlineStr"/>
@@ -14362,44 +14364,42 @@
     <row r="320">
       <c r="A320" s="2" t="inlineStr">
         <is>
-          <t>NTGAZ</t>
+          <t>HOROZ</t>
         </is>
       </c>
       <c r="B320" s="3" t="n">
-        <v>12.68</v>
+        <v>71.75</v>
       </c>
       <c r="C320" s="4" t="n">
-        <v>0.0016</v>
+        <v>0.0235</v>
       </c>
       <c r="D320" s="5" t="n">
-        <v>7760000</v>
+        <v>3740000</v>
       </c>
       <c r="E320" s="4" t="n">
-        <v>0.4</v>
+        <v>0.8178</v>
       </c>
       <c r="F320" s="3" t="n">
-        <v>50.44</v>
-      </c>
-      <c r="G320" s="3" t="n">
-        <v>10.34</v>
-      </c>
+        <v>47.14</v>
+      </c>
+      <c r="G320" s="2" t="inlineStr"/>
       <c r="H320" s="3" t="n">
-        <v>1.74</v>
+        <v>1.73</v>
       </c>
       <c r="I320" s="4" t="n">
-        <v>0.1964</v>
+        <v>-0.0183</v>
       </c>
       <c r="J320" s="4" t="n">
-        <v>4.1859</v>
+        <v>-2.2684</v>
       </c>
       <c r="K320" s="2" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Taşımacılık</t>
         </is>
       </c>
       <c r="L320" s="2" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST KATILIM TEMETTU</t>
+          <t>BIST ULASTIRMA, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M320" s="2" t="inlineStr"/>
@@ -14407,42 +14407,44 @@
     <row r="321">
       <c r="A321" s="6" t="inlineStr">
         <is>
-          <t>DURDO</t>
+          <t>NTGAZ</t>
         </is>
       </c>
       <c r="B321" s="7" t="n">
-        <v>5.12</v>
+        <v>12.68</v>
       </c>
       <c r="C321" s="8" t="n">
-        <v>-0.0173</v>
+        <v>0.0016</v>
       </c>
       <c r="D321" s="9" t="n">
-        <v>4090000</v>
+        <v>7760000</v>
       </c>
       <c r="E321" s="8" t="n">
-        <v>0.8881999999999999</v>
+        <v>0.4</v>
       </c>
       <c r="F321" s="7" t="n">
-        <v>62.78</v>
-      </c>
-      <c r="G321" s="6" t="inlineStr"/>
+        <v>50.44</v>
+      </c>
+      <c r="G321" s="7" t="n">
+        <v>10.34</v>
+      </c>
       <c r="H321" s="7" t="n">
         <v>1.74</v>
       </c>
       <c r="I321" s="8" t="n">
-        <v>-0.1903</v>
+        <v>0.1964</v>
       </c>
       <c r="J321" s="8" t="n">
-        <v>-1.1628</v>
+        <v>4.1859</v>
       </c>
       <c r="K321" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L321" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST İSTANBUL, BIST ANA</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M321" s="6" t="inlineStr"/>
@@ -14450,44 +14452,42 @@
     <row r="322">
       <c r="A322" s="2" t="inlineStr">
         <is>
-          <t>TBORG</t>
+          <t>DURDO</t>
         </is>
       </c>
       <c r="B322" s="3" t="n">
-        <v>136.4</v>
+        <v>5.12</v>
       </c>
       <c r="C322" s="4" t="n">
-        <v>-0.0051</v>
+        <v>-0.0173</v>
       </c>
       <c r="D322" s="5" t="n">
-        <v>223870</v>
+        <v>4090000</v>
       </c>
       <c r="E322" s="4" t="n">
-        <v>0.0501</v>
+        <v>0.8881999999999999</v>
       </c>
       <c r="F322" s="3" t="n">
-        <v>40.13</v>
-      </c>
-      <c r="G322" s="3" t="n">
-        <v>16.19</v>
-      </c>
+        <v>62.78</v>
+      </c>
+      <c r="G322" s="2" t="inlineStr"/>
       <c r="H322" s="3" t="n">
-        <v>1.75</v>
+        <v>1.74</v>
       </c>
       <c r="I322" s="4" t="n">
-        <v>0.1231</v>
+        <v>-0.1903</v>
       </c>
       <c r="J322" s="4" t="n">
-        <v>-1.0574</v>
+        <v>-1.1628</v>
       </c>
       <c r="K322" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L322" s="2" t="inlineStr">
         <is>
-          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST ANA, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST İSTANBUL, BIST ANA</t>
         </is>
       </c>
       <c r="M322" s="2" t="inlineStr"/>
@@ -14495,44 +14495,44 @@
     <row r="323">
       <c r="A323" s="6" t="inlineStr">
         <is>
-          <t>TURGG</t>
+          <t>TBORG</t>
         </is>
       </c>
       <c r="B323" s="7" t="n">
-        <v>30.42</v>
+        <v>136.4</v>
       </c>
       <c r="C323" s="8" t="n">
-        <v>-0.0026</v>
+        <v>-0.0051</v>
       </c>
       <c r="D323" s="9" t="n">
-        <v>661000</v>
+        <v>223870</v>
       </c>
       <c r="E323" s="8" t="n">
-        <v>0.2511</v>
+        <v>0.0501</v>
       </c>
       <c r="F323" s="7" t="n">
-        <v>37.19</v>
+        <v>40.13</v>
       </c>
       <c r="G323" s="7" t="n">
-        <v>17.9</v>
+        <v>16.19</v>
       </c>
       <c r="H323" s="7" t="n">
-        <v>1.76</v>
+        <v>1.75</v>
       </c>
       <c r="I323" s="8" t="n">
-        <v>0.0946</v>
+        <v>0.1231</v>
       </c>
       <c r="J323" s="8" t="n">
-        <v>0.2596</v>
+        <v>-1.0574</v>
       </c>
       <c r="K323" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L323" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M323" s="6" t="inlineStr"/>
@@ -25942,42 +25942,34 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>LILAK</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>34.72</v>
+        <v>39.6</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>-0.0012</v>
+        <v>-0.0365</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>4640000</v>
-      </c>
-      <c r="E588" s="4" t="n">
-        <v>0.3528</v>
-      </c>
+        <v>11700000</v>
+      </c>
+      <c r="E588" s="2" t="inlineStr"/>
       <c r="F588" s="3" t="n">
-        <v>46.16</v>
-      </c>
-      <c r="G588" s="3" t="n">
-        <v>13.72</v>
-      </c>
+        <v>59.52</v>
+      </c>
+      <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
-      <c r="I588" s="4" t="n">
-        <v>0.1029</v>
-      </c>
-      <c r="J588" s="4" t="n">
-        <v>-1.4864</v>
-      </c>
+      <c r="I588" s="2" t="inlineStr"/>
+      <c r="J588" s="2" t="inlineStr"/>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -25985,21 +25977,21 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>40.96</v>
+        <v>16.3</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>0.0039</v>
+        <v>-0.0151</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>4380000</v>
+        <v>30420000</v>
       </c>
       <c r="E589" s="6" t="inlineStr"/>
       <c r="F589" s="7" t="n">
-        <v>50.43</v>
+        <v>45.98</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
@@ -26007,12 +25999,12 @@
       <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26020,38 +26012,34 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>67.15000000000001</v>
+        <v>191.9</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>0.0121</v>
+        <v>-0.0174</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>562280</v>
-      </c>
-      <c r="E590" s="4" t="n">
-        <v>0.3695000000000001</v>
-      </c>
+        <v>5800000</v>
+      </c>
+      <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>54.15</v>
+        <v>55.81</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
       <c r="I590" s="2" t="inlineStr"/>
-      <c r="J590" s="4" t="n">
-        <v>0.1431</v>
-      </c>
+      <c r="J590" s="2" t="inlineStr"/>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26059,60 +26047,62 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>12</v>
+        <v>129.6</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.0345</v>
+        <v>-0.0077</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>498860</v>
+        <v>879570</v>
       </c>
       <c r="E591" s="8" t="n">
-        <v>0.95</v>
+        <v>0.1071</v>
       </c>
       <c r="F591" s="7" t="n">
-        <v>69.81999999999999</v>
+        <v>41.79</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
       <c r="I591" s="8" t="n">
-        <v>-23.6291</v>
+        <v>-3.6635</v>
       </c>
       <c r="J591" s="8" t="n">
-        <v>-0.4678</v>
+        <v>-0.4897</v>
       </c>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L591" s="6" t="inlineStr"/>
+          <t>Perakende satış</t>
+        </is>
+      </c>
+      <c r="L591" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+        </is>
+      </c>
       <c r="M591" s="6" t="inlineStr"/>
     </row>
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>36.38</v>
+        <v>40.96</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>0.0022</v>
+        <v>0.0039</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>23850000</v>
-      </c>
-      <c r="E592" s="4" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>4380000</v>
+      </c>
+      <c r="E592" s="2" t="inlineStr"/>
       <c r="F592" s="3" t="n">
-        <v>68.22</v>
+        <v>50.43</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
@@ -26120,12 +26110,12 @@
       <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L592" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M592" s="2" t="inlineStr"/>
@@ -26133,21 +26123,21 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>2.6</v>
+        <v>17.67</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>-0.0189</v>
+        <v>-0.0172</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>94430000</v>
+        <v>21980000</v>
       </c>
       <c r="E593" s="6" t="inlineStr"/>
       <c r="F593" s="7" t="n">
-        <v>42.83</v>
+        <v>36.71</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
@@ -26160,7 +26150,7 @@
       </c>
       <c r="L593" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M593" s="6" t="inlineStr"/>
@@ -26168,38 +26158,36 @@
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>VKING</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>25.7</v>
+        <v>36.38</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>-0.006999999999999999</v>
+        <v>0.0022</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>527150</v>
+        <v>23850000</v>
       </c>
       <c r="E594" s="4" t="n">
-        <v>0.9698</v>
+        <v>0.2667</v>
       </c>
       <c r="F594" s="3" t="n">
-        <v>45.64</v>
+        <v>68.22</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
       <c r="I594" s="2" t="inlineStr"/>
-      <c r="J594" s="4" t="n">
-        <v>0.6453</v>
-      </c>
+      <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26207,71 +26195,73 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>VKING</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>6.12</v>
+        <v>25.7</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>0.009899999999999999</v>
+        <v>-0.006999999999999999</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>8660000</v>
-      </c>
-      <c r="E595" s="6" t="inlineStr"/>
+        <v>527150</v>
+      </c>
+      <c r="E595" s="8" t="n">
+        <v>0.9698</v>
+      </c>
       <c r="F595" s="7" t="n">
-        <v>54.27</v>
+        <v>45.64</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
       <c r="I595" s="6" t="inlineStr"/>
-      <c r="J595" s="6" t="inlineStr"/>
+      <c r="J595" s="8" t="n">
+        <v>0.6453</v>
+      </c>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L595" s="6" t="inlineStr"/>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
+        </is>
+      </c>
+      <c r="L595" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
+        </is>
+      </c>
       <c r="M595" s="6" t="inlineStr"/>
     </row>
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>129.6</v>
+        <v>2.6</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>-0.0077</v>
+        <v>-0.0189</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>879570</v>
-      </c>
-      <c r="E596" s="4" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>94430000</v>
+      </c>
+      <c r="E596" s="2" t="inlineStr"/>
       <c r="F596" s="3" t="n">
-        <v>41.79</v>
+        <v>42.83</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
-      <c r="I596" s="4" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J596" s="4" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I596" s="2" t="inlineStr"/>
+      <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26279,62 +26269,58 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>5.87</v>
+        <v>12</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0.0731</v>
+        <v>0.0345</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>18100000</v>
+        <v>498860</v>
       </c>
       <c r="E597" s="8" t="n">
-        <v>0.1672</v>
+        <v>0.95</v>
       </c>
       <c r="F597" s="7" t="n">
-        <v>49.01</v>
+        <v>69.81999999999999</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
       <c r="I597" s="8" t="n">
-        <v>-5.3262</v>
+        <v>-23.6291</v>
       </c>
       <c r="J597" s="8" t="n">
-        <v>-4.2562</v>
+        <v>-0.4678</v>
       </c>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L597" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L597" s="6" t="inlineStr"/>
       <c r="M597" s="6" t="inlineStr"/>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>191.9</v>
+        <v>32.18</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.0174</v>
+        <v>0.0255</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>5800000</v>
+        <v>17120000</v>
       </c>
       <c r="E598" s="2" t="inlineStr"/>
       <c r="F598" s="3" t="n">
-        <v>55.81</v>
+        <v>65.51000000000001</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
@@ -26342,12 +26328,12 @@
       <c r="J598" s="2" t="inlineStr"/>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26355,32 +26341,32 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>EKDMR</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>59.85</v>
+        <v>6.12</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>0.0992</v>
-      </c>
-      <c r="D599" s="6" t="inlineStr"/>
+        <v>0.009899999999999999</v>
+      </c>
+      <c r="D599" s="9" t="n">
+        <v>8660000</v>
+      </c>
       <c r="E599" s="6" t="inlineStr"/>
-      <c r="F599" s="6" t="inlineStr"/>
+      <c r="F599" s="7" t="n">
+        <v>54.27</v>
+      </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
       <c r="I599" s="6" t="inlineStr"/>
       <c r="J599" s="6" t="inlineStr"/>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>Enerji-dışı mineraller</t>
-        </is>
-      </c>
-      <c r="L599" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST HALKA ARZ, BIST YILDIZ</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L599" s="6" t="inlineStr"/>
       <c r="M599" s="6" t="inlineStr"/>
     </row>
     <row r="600">
@@ -26417,118 +26403,118 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>70.25</v>
+        <v>13.92</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>0.09939999999999999</v>
+        <v>-0.0029</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>42550</v>
-      </c>
-      <c r="E601" s="8" t="n">
-        <v>0.58</v>
-      </c>
+        <v>19750000</v>
+      </c>
+      <c r="E601" s="6" t="inlineStr"/>
       <c r="F601" s="7" t="n">
-        <v>44.2</v>
+        <v>50.28</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
       <c r="I601" s="6" t="inlineStr"/>
-      <c r="J601" s="8" t="n">
-        <v>0.4928</v>
-      </c>
+      <c r="J601" s="6" t="inlineStr"/>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L601" s="6" t="inlineStr"/>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L601" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+        </is>
+      </c>
       <c r="M601" s="6" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>80.37</v>
+        <v>170.1</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>-0.0042</v>
+        <v>-0.023</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>11050000</v>
+        <v>6070000</v>
       </c>
       <c r="E602" s="2" t="inlineStr"/>
       <c r="F602" s="3" t="n">
-        <v>49.24</v>
+        <v>38.2</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
       <c r="I602" s="2" t="inlineStr"/>
       <c r="J602" s="2" t="inlineStr"/>
-      <c r="K602" s="2" t="inlineStr"/>
-      <c r="L602" s="2" t="inlineStr"/>
+      <c r="K602" s="2" t="inlineStr">
+        <is>
+          <t>Endüstriyel hizmetler</t>
+        </is>
+      </c>
+      <c r="L602" s="2" t="inlineStr">
+        <is>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+        </is>
+      </c>
       <c r="M602" s="2" t="inlineStr"/>
     </row>
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>13.92</v>
+        <v>80.37</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>-0.0029</v>
+        <v>-0.0042</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>19750000</v>
+        <v>11050000</v>
       </c>
       <c r="E603" s="6" t="inlineStr"/>
       <c r="F603" s="7" t="n">
-        <v>50.28</v>
+        <v>49.24</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
       <c r="I603" s="6" t="inlineStr"/>
       <c r="J603" s="6" t="inlineStr"/>
-      <c r="K603" s="6" t="inlineStr">
-        <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L603" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
-        </is>
-      </c>
+      <c r="K603" s="6" t="inlineStr"/>
+      <c r="L603" s="6" t="inlineStr"/>
       <c r="M603" s="6" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>16.49</v>
+        <v>74.05</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>0.005500000000000001</v>
+        <v>-0.0886</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>28260000</v>
+        <v>25520000</v>
       </c>
       <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>48.12</v>
+        <v>67.18000000000001</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
@@ -26536,12 +26522,12 @@
       <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26549,34 +26535,38 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>32.18</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>0.0255</v>
+        <v>0.0121</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>17120000</v>
-      </c>
-      <c r="E605" s="6" t="inlineStr"/>
+        <v>562280</v>
+      </c>
+      <c r="E605" s="8" t="n">
+        <v>0.3695000000000001</v>
+      </c>
       <c r="F605" s="7" t="n">
-        <v>65.51000000000001</v>
+        <v>54.15</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
       <c r="I605" s="6" t="inlineStr"/>
-      <c r="J605" s="6" t="inlineStr"/>
+      <c r="J605" s="8" t="n">
+        <v>0.1431</v>
+      </c>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M605" s="6" t="inlineStr"/>
@@ -26584,21 +26574,21 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>17.67</v>
+        <v>16.49</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>-0.0172</v>
+        <v>0.005500000000000001</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>21980000</v>
+        <v>28260000</v>
       </c>
       <c r="E606" s="2" t="inlineStr"/>
       <c r="F606" s="3" t="n">
-        <v>36.71</v>
+        <v>48.12</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
@@ -26611,7 +26601,7 @@
       </c>
       <c r="L606" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M606" s="2" t="inlineStr"/>
@@ -26619,75 +26609,75 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>2.4</v>
+        <v>70.25</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>0</v>
+        <v>0.09939999999999999</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>16980000</v>
+        <v>42550</v>
       </c>
       <c r="E607" s="8" t="n">
-        <v>1</v>
+        <v>0.58</v>
       </c>
       <c r="F607" s="7" t="n">
-        <v>39.22</v>
+        <v>44.2</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
-      <c r="I607" s="8" t="n">
-        <v>-191.6342</v>
-      </c>
+      <c r="I607" s="6" t="inlineStr"/>
       <c r="J607" s="8" t="n">
-        <v>-0.8093</v>
+        <v>0.4928</v>
       </c>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
-        </is>
-      </c>
-      <c r="L607" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L607" s="6" t="inlineStr"/>
       <c r="M607" s="6" t="inlineStr"/>
     </row>
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B608" s="3" t="n">
-        <v>170.1</v>
+        <v>2.4</v>
       </c>
       <c r="C608" s="4" t="n">
-        <v>-0.023</v>
+        <v>0</v>
       </c>
       <c r="D608" s="5" t="n">
-        <v>6070000</v>
-      </c>
-      <c r="E608" s="2" t="inlineStr"/>
+        <v>16980000</v>
+      </c>
+      <c r="E608" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="F608" s="3" t="n">
-        <v>38.2</v>
+        <v>39.22</v>
       </c>
       <c r="G608" s="2" t="inlineStr"/>
       <c r="H608" s="2" t="inlineStr"/>
-      <c r="I608" s="2" t="inlineStr"/>
-      <c r="J608" s="2" t="inlineStr"/>
+      <c r="I608" s="4" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J608" s="4" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K608" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L608" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M608" s="2" t="inlineStr"/>
@@ -26695,34 +26685,40 @@
     <row r="609">
       <c r="A609" s="6" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B609" s="7" t="n">
-        <v>74.05</v>
+        <v>5.87</v>
       </c>
       <c r="C609" s="8" t="n">
-        <v>-0.0886</v>
+        <v>0.0731</v>
       </c>
       <c r="D609" s="9" t="n">
-        <v>25520000</v>
-      </c>
-      <c r="E609" s="6" t="inlineStr"/>
+        <v>18100000</v>
+      </c>
+      <c r="E609" s="8" t="n">
+        <v>0.1672</v>
+      </c>
       <c r="F609" s="7" t="n">
-        <v>67.18000000000001</v>
+        <v>49.01</v>
       </c>
       <c r="G609" s="6" t="inlineStr"/>
       <c r="H609" s="6" t="inlineStr"/>
-      <c r="I609" s="6" t="inlineStr"/>
-      <c r="J609" s="6" t="inlineStr"/>
+      <c r="I609" s="8" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J609" s="8" t="n">
+        <v>-4.2562</v>
+      </c>
       <c r="K609" s="6" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L609" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M609" s="6" t="inlineStr"/>
@@ -26730,21 +26726,23 @@
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B610" s="3" t="n">
-        <v>39.6</v>
+        <v>245</v>
       </c>
       <c r="C610" s="4" t="n">
-        <v>-0.0365</v>
+        <v>0.0298</v>
       </c>
       <c r="D610" s="5" t="n">
-        <v>11700000</v>
-      </c>
-      <c r="E610" s="2" t="inlineStr"/>
+        <v>9560</v>
+      </c>
+      <c r="E610" s="4" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F610" s="3" t="n">
-        <v>59.52</v>
+        <v>50.37</v>
       </c>
       <c r="G610" s="2" t="inlineStr"/>
       <c r="H610" s="2" t="inlineStr"/>
@@ -26752,47 +26750,39 @@
       <c r="J610" s="2" t="inlineStr"/>
       <c r="K610" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L610" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L610" s="2" t="inlineStr"/>
       <c r="M610" s="2" t="inlineStr"/>
     </row>
     <row r="611">
       <c r="A611" s="6" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>EKDMR</t>
         </is>
       </c>
       <c r="B611" s="7" t="n">
-        <v>16.3</v>
+        <v>59.85</v>
       </c>
       <c r="C611" s="8" t="n">
-        <v>-0.0151</v>
-      </c>
-      <c r="D611" s="9" t="n">
-        <v>30420000</v>
-      </c>
+        <v>0.0992</v>
+      </c>
+      <c r="D611" s="6" t="inlineStr"/>
       <c r="E611" s="6" t="inlineStr"/>
-      <c r="F611" s="7" t="n">
-        <v>45.98</v>
-      </c>
+      <c r="F611" s="6" t="inlineStr"/>
       <c r="G611" s="6" t="inlineStr"/>
       <c r="H611" s="6" t="inlineStr"/>
       <c r="I611" s="6" t="inlineStr"/>
       <c r="J611" s="6" t="inlineStr"/>
       <c r="K611" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Enerji-dışı mineraller</t>
         </is>
       </c>
       <c r="L611" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST HALKA ARZ, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M611" s="6" t="inlineStr"/>
@@ -26800,34 +26790,44 @@
     <row r="612">
       <c r="A612" s="2" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>LILAK</t>
         </is>
       </c>
       <c r="B612" s="3" t="n">
-        <v>245</v>
+        <v>34.72</v>
       </c>
       <c r="C612" s="4" t="n">
-        <v>0.0298</v>
+        <v>-0.0012</v>
       </c>
       <c r="D612" s="5" t="n">
-        <v>9560</v>
+        <v>4640000</v>
       </c>
       <c r="E612" s="4" t="n">
-        <v>0.2578</v>
+        <v>0.3528</v>
       </c>
       <c r="F612" s="3" t="n">
-        <v>50.37</v>
-      </c>
-      <c r="G612" s="2" t="inlineStr"/>
+        <v>46.16</v>
+      </c>
+      <c r="G612" s="3" t="n">
+        <v>13.72</v>
+      </c>
       <c r="H612" s="2" t="inlineStr"/>
-      <c r="I612" s="2" t="inlineStr"/>
-      <c r="J612" s="2" t="inlineStr"/>
+      <c r="I612" s="4" t="n">
+        <v>0.1029</v>
+      </c>
+      <c r="J612" s="4" t="n">
+        <v>-1.4864</v>
+      </c>
       <c r="K612" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L612" s="2" t="inlineStr"/>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
+        </is>
+      </c>
+      <c r="L612" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
+        </is>
+      </c>
       <c r="M612" s="2" t="inlineStr"/>
     </row>
   </sheetData>
@@ -26852,7 +26852,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>28.05.2026 05:27</t>
+          <t>28.05.2026 18:22</t>
         </is>
       </c>
     </row>

</xml_diff>